<commit_message>
fix missing average gpa for 'Aerospace Engr
</commit_message>
<xml_diff>
--- a/data/avergeGPA.xlsx
+++ b/data/avergeGPA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brand\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\brand\Downloads\Software Eng\Personal Projects\Masters Project\CPPMajorScraper\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2D5DCFDA-95A2-4F01-A99E-12011048AB96}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8FC75C57-E2E8-43CC-B849-11D6E04AC7DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3465" yWindow="2790" windowWidth="21600" windowHeight="11295" xr2:uid="{07FF3B72-D4BA-43C3-8CAE-9E312F5D43E1}"/>
+    <workbookView xWindow="735" yWindow="735" windowWidth="21600" windowHeight="11295" xr2:uid="{07FF3B72-D4BA-43C3-8CAE-9E312F5D43E1}"/>
   </bookViews>
   <sheets>
     <sheet name="FTS Avg GPA by Major" sheetId="6" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19019" uniqueCount="257">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19018" uniqueCount="257">
   <si>
     <t>College</t>
   </si>
@@ -9777,7 +9777,7 @@
         <v>3.33</v>
       </c>
     </row>
-    <row r="401" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A401" t="s">
         <v>42</v>
       </c>
@@ -9797,7 +9797,7 @@
         <v>2.27</v>
       </c>
     </row>
-    <row r="402" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A402" t="s">
         <v>42</v>
       </c>
@@ -9817,7 +9817,7 @@
         <v>2.87</v>
       </c>
     </row>
-    <row r="403" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A403" t="s">
         <v>42</v>
       </c>
@@ -9837,7 +9837,7 @@
         <v>3.14</v>
       </c>
     </row>
-    <row r="404" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A404" t="s">
         <v>42</v>
       </c>
@@ -9857,7 +9857,7 @@
         <v>2.92</v>
       </c>
     </row>
-    <row r="405" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A405" t="s">
         <v>42</v>
       </c>
@@ -9877,7 +9877,7 @@
         <v>2.56</v>
       </c>
     </row>
-    <row r="406" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A406" t="s">
         <v>42</v>
       </c>
@@ -9897,7 +9897,7 @@
         <v>2.96</v>
       </c>
     </row>
-    <row r="407" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A407" t="s">
         <v>42</v>
       </c>
@@ -9917,7 +9917,7 @@
         <v>3.15</v>
       </c>
     </row>
-    <row r="408" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A408" t="s">
         <v>42</v>
       </c>
@@ -9937,7 +9937,7 @@
         <v>2.89</v>
       </c>
     </row>
-    <row r="409" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A409" t="s">
         <v>42</v>
       </c>
@@ -9957,7 +9957,7 @@
         <v>2.96</v>
       </c>
     </row>
-    <row r="410" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A410" t="s">
         <v>42</v>
       </c>
@@ -9977,7 +9977,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="411" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A411" t="s">
         <v>42</v>
       </c>
@@ -9997,7 +9997,7 @@
         <v>3.17</v>
       </c>
     </row>
-    <row r="412" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A412" t="s">
         <v>42</v>
       </c>
@@ -10017,7 +10017,7 @@
         <v>2.99</v>
       </c>
     </row>
-    <row r="413" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A413" t="s">
         <v>42</v>
       </c>
@@ -10037,7 +10037,7 @@
         <v>2.86</v>
       </c>
     </row>
-    <row r="414" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A414" t="s">
         <v>42</v>
       </c>
@@ -10057,7 +10057,7 @@
         <v>3.01</v>
       </c>
     </row>
-    <row r="415" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A415" t="s">
         <v>42</v>
       </c>
@@ -10077,7 +10077,7 @@
         <v>3.19</v>
       </c>
     </row>
-    <row r="416" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A416" t="s">
         <v>42</v>
       </c>
@@ -10097,7 +10097,7 @@
         <v>3.03</v>
       </c>
     </row>
-    <row r="417" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A417" t="s">
         <v>42</v>
       </c>
@@ -10117,7 +10117,7 @@
         <v>2.4900000000000002</v>
       </c>
     </row>
-    <row r="418" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A418" t="s">
         <v>42</v>
       </c>
@@ -10137,7 +10137,7 @@
         <v>3.05</v>
       </c>
     </row>
-    <row r="419" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
         <v>42</v>
       </c>
@@ -10157,7 +10157,7 @@
         <v>3.21</v>
       </c>
     </row>
-    <row r="420" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A420" t="s">
         <v>42</v>
       </c>
@@ -10177,7 +10177,7 @@
         <v>3.07</v>
       </c>
     </row>
-    <row r="421" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A421" t="s">
         <v>42</v>
       </c>
@@ -10197,7 +10197,7 @@
         <v>2.37</v>
       </c>
     </row>
-    <row r="422" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A422" t="s">
         <v>42</v>
       </c>
@@ -10217,7 +10217,7 @@
         <v>3.1</v>
       </c>
     </row>
-    <row r="423" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A423" t="s">
         <v>42</v>
       </c>
@@ -10237,7 +10237,7 @@
         <v>3.25</v>
       </c>
     </row>
-    <row r="424" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A424" t="s">
         <v>42</v>
       </c>
@@ -10257,7 +10257,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="425" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A425" t="s">
         <v>42</v>
       </c>
@@ -10277,7 +10277,7 @@
         <v>2.25</v>
       </c>
     </row>
-    <row r="426" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A426" t="s">
         <v>42</v>
       </c>
@@ -10297,7 +10297,7 @@
         <v>3.14</v>
       </c>
     </row>
-    <row r="427" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A427" t="s">
         <v>42</v>
       </c>
@@ -10317,7 +10317,7 @@
         <v>3.23</v>
       </c>
     </row>
-    <row r="428" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
       <c r="A428" t="s">
         <v>42</v>
       </c>
@@ -10857,7 +10857,7 @@
         <v>2.86</v>
       </c>
     </row>
-    <row r="455" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A455" t="s">
         <v>45</v>
       </c>
@@ -10877,7 +10877,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="456" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A456" t="s">
         <v>45</v>
       </c>
@@ -10897,7 +10897,7 @@
         <v>3.07</v>
       </c>
     </row>
-    <row r="457" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A457" t="s">
         <v>45</v>
       </c>
@@ -10917,7 +10917,7 @@
         <v>3.07</v>
       </c>
     </row>
-    <row r="458" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A458" t="s">
         <v>45</v>
       </c>
@@ -10937,7 +10937,7 @@
         <v>3.08</v>
       </c>
     </row>
-    <row r="459" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A459" t="s">
         <v>45</v>
       </c>
@@ -10957,7 +10957,7 @@
         <v>2.4900000000000002</v>
       </c>
     </row>
-    <row r="460" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A460" t="s">
         <v>45</v>
       </c>
@@ -10977,7 +10977,7 @@
         <v>3.15</v>
       </c>
     </row>
-    <row r="461" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A461" t="s">
         <v>45</v>
       </c>
@@ -10997,7 +10997,7 @@
         <v>3.11</v>
       </c>
     </row>
-    <row r="462" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A462" t="s">
         <v>45</v>
       </c>
@@ -11017,7 +11017,7 @@
         <v>3.14</v>
       </c>
     </row>
-    <row r="463" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A463" t="s">
         <v>45</v>
       </c>
@@ -11037,7 +11037,7 @@
         <v>2.86</v>
       </c>
     </row>
-    <row r="464" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A464" t="s">
         <v>45</v>
       </c>
@@ -11057,7 +11057,7 @@
         <v>3.26</v>
       </c>
     </row>
-    <row r="465" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A465" t="s">
         <v>45</v>
       </c>
@@ -11077,7 +11077,7 @@
         <v>3.2</v>
       </c>
     </row>
-    <row r="466" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A466" t="s">
         <v>45</v>
       </c>
@@ -11097,7 +11097,7 @@
         <v>3.26</v>
       </c>
     </row>
-    <row r="467" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A467" t="s">
         <v>45</v>
       </c>
@@ -11117,7 +11117,7 @@
         <v>2.86</v>
       </c>
     </row>
-    <row r="468" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A468" t="s">
         <v>45</v>
       </c>
@@ -11137,7 +11137,7 @@
         <v>3.28</v>
       </c>
     </row>
-    <row r="469" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A469" t="s">
         <v>45</v>
       </c>
@@ -11157,7 +11157,7 @@
         <v>3.24</v>
       </c>
     </row>
-    <row r="470" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A470" t="s">
         <v>45</v>
       </c>
@@ -11177,7 +11177,7 @@
         <v>3.22</v>
       </c>
     </row>
-    <row r="471" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A471" t="s">
         <v>45</v>
       </c>
@@ -11197,7 +11197,7 @@
         <v>2.96</v>
       </c>
     </row>
-    <row r="472" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A472" t="s">
         <v>45</v>
       </c>
@@ -11217,7 +11217,7 @@
         <v>3.28</v>
       </c>
     </row>
-    <row r="473" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A473" t="s">
         <v>45</v>
       </c>
@@ -11237,7 +11237,7 @@
         <v>3.24</v>
       </c>
     </row>
-    <row r="474" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A474" t="s">
         <v>45</v>
       </c>
@@ -11257,7 +11257,7 @@
         <v>3.28</v>
       </c>
     </row>
-    <row r="475" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A475" t="s">
         <v>45</v>
       </c>
@@ -11277,7 +11277,7 @@
         <v>2.78</v>
       </c>
     </row>
-    <row r="476" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A476" t="s">
         <v>45</v>
       </c>
@@ -11297,7 +11297,7 @@
         <v>3.32</v>
       </c>
     </row>
-    <row r="477" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A477" t="s">
         <v>45</v>
       </c>
@@ -11317,7 +11317,7 @@
         <v>3.26</v>
       </c>
     </row>
-    <row r="478" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A478" t="s">
         <v>45</v>
       </c>
@@ -11337,7 +11337,7 @@
         <v>3.28</v>
       </c>
     </row>
-    <row r="479" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A479" t="s">
         <v>45</v>
       </c>
@@ -11357,7 +11357,7 @@
         <v>2.65</v>
       </c>
     </row>
-    <row r="480" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A480" t="s">
         <v>45</v>
       </c>
@@ -11377,7 +11377,7 @@
         <v>3.28</v>
       </c>
     </row>
-    <row r="481" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A481" t="s">
         <v>45</v>
       </c>
@@ -11397,7 +11397,7 @@
         <v>3.28</v>
       </c>
     </row>
-    <row r="482" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A482" t="s">
         <v>45</v>
       </c>
@@ -31075,11 +31075,6 @@
       </c>
       <c r="F1465" s="1">
         <v>3.11</v>
-      </c>
-    </row>
-    <row r="1466" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
-      <c r="C1466" t="s">
-        <v>46</v>
       </c>
     </row>
     <row r="1467" spans="1:6" hidden="1" x14ac:dyDescent="0.25">
@@ -34061,7 +34056,7 @@
   <autoFilter ref="A1:F1608" xr:uid="{0D7C1E1B-5F58-468B-805D-10DFF4D4E856}">
     <filterColumn colId="2">
       <filters>
-        <filter val="Early Childhood Teaching, Integrated Teacher Education Program Education Specialist: Extensive Support Needs, Integrated Teacher Education Program Education Specialist: Mild to Moderate Support Needs, Multilingual Teaching, Non-Teaching, Pre-K to Grade 3"/>
+        <filter val="Aerospace Engineering"/>
       </filters>
     </filterColumn>
     <filterColumn colId="3">
@@ -79132,12 +79127,14 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b53979b8-abe1-41f1-9197-83890245525e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="d205d236-17e5-47e3-949e-9f7ee3bba6b3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -79384,20 +79381,27 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b53979b8-abe1-41f1-9197-83890245525e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="d205d236-17e5-47e3-949e-9f7ee3bba6b3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA016A25-0EEE-4AE4-ACBA-77CF8DE5B84B}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97D720EC-5EC5-4627-AB66-D51636E69EBC}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="d205d236-17e5-47e3-949e-9f7ee3bba6b3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="b53979b8-abe1-41f1-9197-83890245525e"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -79422,18 +79426,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{97D720EC-5EC5-4627-AB66-D51636E69EBC}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA016A25-0EEE-4AE4-ACBA-77CF8DE5B84B}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="d205d236-17e5-47e3-949e-9f7ee3bba6b3"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="b53979b8-abe1-41f1-9197-83890245525e"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>